<commit_message>
Update TRUST Sheet core message on About Me and dashboard
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DDRxLznxQFLEsk2zkizz32
</commit_message>
<xml_diff>
--- a/icyber/TRUST-Tracker-Freedom-Edition.xlsx
+++ b/icyber/TRUST-Tracker-Freedom-Edition.xlsx
@@ -145,7 +145,7 @@
     <t xml:space="preserve">Head to the How to Use tab. In about 20 minutes you'll have your first financial snapshot. You don't need everything figured out today. You just need somewhere meaningful to start.</t>
   </si>
   <si>
-    <t xml:space="preserve">You work hard to build a better life. Your money should help you live it, not just keep you working for it.</t>
+    <t xml:space="preserve">Financial freedom isn't about quitting your 9–5. It's about using your career as the engine to fuel your financial independence, build multiple income streams, and create the freedom to spend more time with the people you love.</t>
   </si>
   <si>
     <t xml:space="preserve">Build your options without quitting your 9–5.  Know your money. Build your wealth. Reclaim your time.
@@ -851,7 +851,7 @@
     <t xml:space="preserve">6 · Free to choose: extra income ≥ needs</t>
   </si>
   <si>
-    <t xml:space="preserve">Your money should help you live the life you work for, not just keep you working for it. Keep your first hour, and keep going. — Liliane</t>
+    <t xml:space="preserve">Your career is the engine. Keep your first hour, and keep going. — Liliane</t>
   </si>
   <si>
     <t xml:space="preserve">Educational tool. Not financial advice.</t>
@@ -1982,7 +1982,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B30" s="8" t="s">
         <v>23</v>
       </c>

</xml_diff>

<commit_message>
Intro: drop emoji, add who Liliane is and why she can speak to this
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DDRxLznxQFLEsk2zkizz32
</commit_message>
<xml_diff>
--- a/icyber/TRUST-Tracker-Freedom-Edition.xlsx
+++ b/icyber/TRUST-Tracker-Freedom-Edition.xlsx
@@ -74,12 +74,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="293">
-  <si>
-    <t xml:space="preserve">Hey, I'm Liliane. 👋</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="294">
+  <si>
+    <t xml:space="preserve">Hey, I'm Liliane.</t>
   </si>
   <si>
     <t xml:space="preserve">You work hard for your money. But is it creating the life you're working so hard for?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I'm a full-time cybersecurity consultant at a Big Four firm. I work a demanding job, and I'm also caring for my mum after her cerebral haemorrhage. I paid off €20,000 of debt and I'm building wealth beside my career with the same system I share here. I don't teach this from the outside. I live it every week.</t>
   </si>
   <si>
     <t xml:space="preserve">You have a demanding career, bills to pay and people who depend on you. You earn a respectable income. Yet despite everything you do, you don't always feel as financially secure or independent as you thought you would.</t>
@@ -1009,6 +1012,14 @@
       <charset val="1"/>
     </font>
     <font>
+      <b val="true"/>
+      <sz val="10.5"/>
+      <color rgb="FF134E4E"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <sz val="10.5"/>
       <color rgb="FF213534"/>
       <name val="Arial"/>
@@ -1035,14 +1046,6 @@
       <i val="true"/>
       <sz val="10.5"/>
       <color rgb="FF6E8180"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="10.5"/>
-      <color rgb="FF134E4E"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -1220,14 +1223,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE8F4F2"/>
-        <bgColor rgb="FFF2F8F7"/>
+        <fgColor rgb="FFF2F8F7"/>
+        <bgColor rgb="FFE8F4F2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF2F8F7"/>
-        <bgColor rgb="FFE8F4F2"/>
+        <fgColor rgb="FFE8F4F2"/>
+        <bgColor rgb="FFF2F8F7"/>
       </patternFill>
     </fill>
     <fill>
@@ -1305,15 +1308,15 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1321,11 +1324,11 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1361,7 +1364,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1385,183 +1388,183 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="165" fontId="24" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="26" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="20" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="20" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="28" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="22" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="26" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="22" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="20" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="22" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="28" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="20" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="28" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="24" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="29" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="165" fontId="24" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="17" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="26" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="17" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="20" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="170" fontId="24" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="166" fontId="20" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="28" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="22" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="26" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="170" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="170" fontId="22" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="170" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="20" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="22" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="28" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="170" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="170" fontId="20" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="170" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="28" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="170" fontId="24" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="29" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="24" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="17" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="17" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="20" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="170" fontId="24" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="20" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="170" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1859,7 +1862,7 @@
     <tabColor rgb="FF9E1B5E"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B2:B33"/>
+  <dimension ref="B2:B34"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
@@ -1882,119 +1885,124 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="48.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="3" t="s">
+    <row r="7" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B7" s="5" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B8" s="3" t="s">
+    <row r="8" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B8" s="4" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B10" s="5" t="s">
+    <row r="9" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B9" s="4" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="6" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="4" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B13" s="3" t="s">
+      <c r="B13" s="4" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="4" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B15" s="3" t="s">
+      <c r="B15" s="4" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B16" s="6" t="s">
+      <c r="B16" s="4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B18" s="5" t="s">
+    <row r="17" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B17" s="7" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B19" s="7" t="s">
+    <row r="19" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B19" s="6" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B20" s="3" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B21" s="3" t="s">
+      <c r="B21" s="4" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B22" s="3" t="s">
+      <c r="B22" s="4" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B23" s="3" t="s">
+      <c r="B23" s="4" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B24" s="3" t="s">
+      <c r="B24" s="4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B25" s="6" t="s">
+    <row r="25" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B25" s="4" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B27" s="5" t="s">
+    <row r="26" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B26" s="7" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B28" s="3" t="s">
+    <row r="28" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B28" s="6" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B30" s="8" t="s">
+    <row r="29" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B29" s="4" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B31" s="9" t="s">
+    <row r="31" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B31" s="8" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B33" s="10" t="s">
+    <row r="32" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B32" s="9" t="s">
         <v>25</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B34" s="10" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -2029,7 +2037,7 @@
   <sheetData>
     <row r="2" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="11" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C2" s="11"/>
       <c r="D2" s="11"/>
@@ -2044,7 +2052,7 @@
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="12" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C3" s="12"/>
       <c r="D3" s="12"/>
@@ -2059,42 +2067,42 @@
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="19" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C5" s="19" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="D5" s="19" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="E5" s="19" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="F5" s="19" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="G5" s="19" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="H5" s="19" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="I5" s="19" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="J5" s="19" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="K5" s="19" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="L5" s="19" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="20" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C6" s="21" t="n">
         <v>2500</v>
@@ -2127,12 +2135,12 @@
         <v>Level 1 · Stable</v>
       </c>
       <c r="L6" s="20" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="20" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C7" s="21" t="n">
         <v>2560</v>
@@ -2165,7 +2173,7 @@
         <v>Level 1 · Stable</v>
       </c>
       <c r="L7" s="20" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2413,160 +2421,160 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="E1" s="0" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="F1" s="0" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
   </sheetData>
@@ -2597,51 +2605,51 @@
   <sheetData>
     <row r="2" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="11" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C2" s="11"/>
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="12" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C3" s="12"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="13" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="14" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="14" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="14" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="14" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2650,23 +2658,23 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="13" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="14" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C12" s="15" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="14" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C13" s="15" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2675,31 +2683,31 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="13" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="16" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C16" s="15" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="14" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C17" s="15" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="17" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C18" s="15" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2709,7 +2717,7 @@
     <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B20" s="14"/>
       <c r="C20" s="15" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -2746,7 +2754,7 @@
   <sheetData>
     <row r="2" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="11" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C2" s="11"/>
       <c r="D2" s="11"/>
@@ -2755,7 +2763,7 @@
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="12" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C3" s="12"/>
       <c r="D3" s="12"/>
@@ -2764,26 +2772,26 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="18" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="19" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E6" s="19" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="20" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C7" s="20" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E7" s="21" t="n">
         <v>2500</v>
@@ -2791,10 +2799,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="20" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C8" s="20" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E8" s="22" t="n">
         <f aca="false">'Income Streams'!G23</f>
@@ -2803,10 +2811,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="20" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C9" s="20" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E9" s="21" t="n">
         <v>0</v>
@@ -2829,7 +2837,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="14" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E13" s="23" t="n">
         <f aca="false">SUM(E7:E12)</f>
@@ -2838,52 +2846,52 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="18" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="19" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C16" s="19" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D16" s="19" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E16" s="19" t="s">
+        <v>56</v>
+      </c>
+      <c r="F16" s="19" t="s">
         <v>55</v>
-      </c>
-      <c r="F16" s="19" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="20" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C17" s="20" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D17" s="20" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E17" s="21" t="n">
         <v>900</v>
       </c>
       <c r="F17" s="20" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="20" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C18" s="20" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D18" s="20" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E18" s="21" t="n">
         <v>140</v>
@@ -2892,13 +2900,13 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="20" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C19" s="20" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D19" s="20" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E19" s="21" t="n">
         <v>320</v>
@@ -2907,13 +2915,13 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="20" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C20" s="20" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D20" s="20" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E20" s="21" t="n">
         <v>90</v>
@@ -2922,13 +2930,13 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="20" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C21" s="20" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D21" s="20" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E21" s="21" t="n">
         <v>80</v>
@@ -2937,13 +2945,13 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="20" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C22" s="20" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D22" s="20" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E22" s="21" t="n">
         <v>150</v>
@@ -2952,13 +2960,13 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="20" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C23" s="20" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D23" s="20" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E23" s="21" t="n">
         <v>60</v>
@@ -2967,13 +2975,13 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="20" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C24" s="20" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D24" s="20" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E24" s="21" t="n">
         <v>45</v>
@@ -2982,13 +2990,13 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="20" t="s">
+        <v>85</v>
+      </c>
+      <c r="C25" s="20" t="s">
+        <v>86</v>
+      </c>
+      <c r="D25" s="20" t="s">
         <v>84</v>
-      </c>
-      <c r="C25" s="20" t="s">
-        <v>85</v>
-      </c>
-      <c r="D25" s="20" t="s">
-        <v>83</v>
       </c>
       <c r="E25" s="21" t="n">
         <v>120</v>
@@ -2997,13 +3005,13 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="20" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C26" s="20" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D26" s="20" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E26" s="21" t="n">
         <v>100</v>
@@ -3222,7 +3230,7 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B58" s="14" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E58" s="23" t="n">
         <f aca="false">SUMIF(D17:D56,"Need",E17:E56)</f>
@@ -3231,7 +3239,7 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B59" s="14" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E59" s="23" t="n">
         <f aca="false">SUMIF(D17:D56,"Want",E17:E56)</f>
@@ -3240,7 +3248,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B60" s="24" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E60" s="25" t="n">
         <f aca="false">SUMIF(C17:C56,"Caregiving",E17:E56)</f>
@@ -3249,7 +3257,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B61" s="26" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="E61" s="27" t="n">
         <f aca="false">SUM(E17:E56)-E58-E59</f>
@@ -3258,7 +3266,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B62" s="28" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E62" s="29" t="n">
         <f aca="false">E13-E58-E59</f>
@@ -3267,7 +3275,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B63" s="28" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="E63" s="30" t="n">
         <f aca="false">IF(E13&gt;0,E62/E13,0)</f>
@@ -3319,7 +3327,7 @@
   <sheetData>
     <row r="2" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="11" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C2" s="11"/>
       <c r="D2" s="11"/>
@@ -3329,7 +3337,7 @@
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="12" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C3" s="12"/>
       <c r="D3" s="12"/>
@@ -3339,33 +3347,33 @@
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="19" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C5" s="19" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D5" s="19" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E5" s="19" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F5" s="19" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="G5" s="19" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="20" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C6" s="21" t="n">
         <v>13</v>
       </c>
       <c r="D6" s="20" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E6" s="21" t="n">
         <v>0</v>
@@ -3375,18 +3383,18 @@
         <v>13</v>
       </c>
       <c r="G6" s="20" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="20" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C7" s="21" t="n">
         <v>35</v>
       </c>
       <c r="D7" s="20" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E7" s="21" t="n">
         <v>15</v>
@@ -3396,18 +3404,18 @@
         <v>20</v>
       </c>
       <c r="G7" s="20" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="20" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C8" s="21" t="n">
         <v>40</v>
       </c>
       <c r="D8" s="20" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E8" s="21" t="n">
         <v>25</v>
@@ -3417,18 +3425,18 @@
         <v>15</v>
       </c>
       <c r="G8" s="20" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="20" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C9" s="21" t="n">
         <v>3</v>
       </c>
       <c r="D9" s="20" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E9" s="21" t="n">
         <v>3</v>
@@ -3672,7 +3680,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="14" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F32" s="29" t="n">
         <f aca="false">SUM(F6:F30)</f>
@@ -3681,7 +3689,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="14" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F33" s="29" t="n">
         <f aca="false">F32*12</f>
@@ -3690,7 +3698,7 @@
     </row>
     <row r="35" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B35" s="32" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C35" s="32"/>
       <c r="D35" s="32"/>
@@ -3742,7 +3750,7 @@
   <sheetData>
     <row r="2" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="11" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C2" s="11"/>
       <c r="D2" s="11"/>
@@ -3754,7 +3762,7 @@
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="12" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C3" s="12"/>
       <c r="D3" s="12"/>
@@ -3766,33 +3774,33 @@
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="19" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C5" s="19" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D5" s="19" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E5" s="19" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F5" s="19" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="G5" s="19" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H5" s="19" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="I5" s="19" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="20" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C6" s="21" t="n">
         <v>1500</v>
@@ -3821,7 +3829,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="20" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C7" s="21" t="n">
         <v>0</v>
@@ -4002,14 +4010,14 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="14" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C17" s="37" t="n">
         <f aca="false">SUM(C6:C15)</f>
         <v>1500</v>
       </c>
       <c r="D17" s="32" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E17" s="32"/>
       <c r="F17" s="32"/>
@@ -4019,7 +4027,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="14" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C18" s="38" t="n">
         <f aca="false">SUM(G6:G15)</f>
@@ -4034,7 +4042,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="14" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C19" s="37" t="n">
         <f aca="false">C18*12</f>
@@ -4049,27 +4057,27 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="18" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B23" s="19" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C23" s="19" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B24" s="15" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C24" s="39" t="n">
         <f aca="false">'T · Track'!E7</f>
         <v>2500</v>
       </c>
       <c r="D24" s="32" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E24" s="32"/>
       <c r="F24" s="32"/>
@@ -4079,7 +4087,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="15" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C25" s="40" t="n">
         <v>39</v>
@@ -4093,7 +4101,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="15" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C26" s="40" t="n">
         <v>4</v>
@@ -4107,7 +4115,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="15" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C27" s="40" t="n">
         <v>5</v>
@@ -4121,7 +4129,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="41" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C28" s="42" t="n">
         <f aca="false">(N(C25)+N(C26)+N(C27))*52/12</f>
@@ -4136,14 +4144,14 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B29" s="28" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C29" s="43" t="n">
         <f aca="false">IF(C28&gt;0,C24/C28,0)</f>
         <v>12.0192307692308</v>
       </c>
       <c r="D29" s="32" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E29" s="32"/>
       <c r="F29" s="32"/>
@@ -4153,7 +4161,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="15" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C30" s="44" t="n">
         <v>21</v>
@@ -4167,7 +4175,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="28" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C31" s="29" t="n">
         <f aca="false">C29*N(C30)</f>
@@ -4218,7 +4226,7 @@
   <sheetData>
     <row r="2" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="11" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C2" s="11"/>
       <c r="D2" s="11"/>
@@ -4228,7 +4236,7 @@
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="12" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C3" s="12"/>
       <c r="D3" s="12"/>
@@ -4238,27 +4246,27 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="18" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="19" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="15" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C7" s="39" t="n">
         <f aca="false">'T · Track'!E58</f>
         <v>1740</v>
       </c>
       <c r="D7" s="32" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="E7" s="32"/>
       <c r="F7" s="32"/>
@@ -4266,7 +4274,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="15" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C8" s="44" t="n">
         <v>3</v>
@@ -4278,7 +4286,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="41" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C9" s="45" t="n">
         <f aca="false">C7</f>
@@ -4291,7 +4299,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="41" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C10" s="23" t="n">
         <f aca="false">C7*N(C8)</f>
@@ -4304,7 +4312,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="15" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C11" s="21" t="n">
         <v>1200</v>
@@ -4312,7 +4320,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="28" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C12" s="30" t="n">
         <f aca="false">IF(C10&gt;0,MIN(1,N(C11)/C10),0)</f>
@@ -4321,7 +4329,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="15" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C13" s="21" t="n">
         <v>250</v>
@@ -4329,7 +4337,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="41" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C14" s="35" t="n">
         <f aca="false">IF(N(C11)&gt;=C10,"Done ✓",IF(N(C13)&gt;0,ROUNDUP((C10-N(C11))/C13,0),"Add a transfer"))</f>
@@ -4338,32 +4346,32 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="18" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B18" s="19" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C18" s="19" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D18" s="19" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="E18" s="19" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F18" s="19" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="G18" s="19" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="20" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C19" s="21" t="n">
         <v>1500</v>
@@ -4385,7 +4393,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="20" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C20" s="21" t="n">
         <v>600</v>
@@ -4407,7 +4415,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="20" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C21" s="21" t="n">
         <v>1800</v>
@@ -4527,7 +4535,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="41" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E30" s="23" t="n">
         <f aca="false">SUM(E19:E28)</f>
@@ -4536,7 +4544,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="28" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="E31" s="29" t="n">
         <f aca="false">N(C13)+E30</f>
@@ -4545,7 +4553,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="14" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="E32" s="23" t="n">
         <f aca="false">'T · Track'!E62-E31</f>
@@ -4554,7 +4562,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B33" s="32" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C33" s="32"/>
       <c r="D33" s="32"/>
@@ -4596,7 +4604,7 @@
   <sheetData>
     <row r="2" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="11" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C2" s="11"/>
       <c r="D2" s="11"/>
@@ -4604,7 +4612,7 @@
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="12" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C3" s="12"/>
       <c r="D3" s="12"/>
@@ -4612,21 +4620,21 @@
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="19" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C5" s="19" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D5" s="19" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="E5" s="19" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="20" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C6" s="40" t="n">
         <v>49</v>
@@ -4635,12 +4643,12 @@
         <v>52</v>
       </c>
       <c r="E6" s="20" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="20" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C7" s="40" t="n">
         <v>43</v>
@@ -4649,12 +4657,12 @@
         <v>40</v>
       </c>
       <c r="E7" s="20" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="20" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C8" s="40" t="n">
         <v>5</v>
@@ -4666,7 +4674,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="20" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C9" s="40" t="n">
         <v>10</v>
@@ -4675,12 +4683,12 @@
         <v>10</v>
       </c>
       <c r="E9" s="20" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="20" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C10" s="40" t="n">
         <v>10</v>
@@ -4689,12 +4697,12 @@
         <v>8</v>
       </c>
       <c r="E10" s="20" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="20" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C11" s="40" t="n">
         <v>12</v>
@@ -4703,12 +4711,12 @@
         <v>16</v>
       </c>
       <c r="E11" s="20" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="20" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C12" s="40" t="n">
         <v>3</v>
@@ -4717,12 +4725,12 @@
         <v>4</v>
       </c>
       <c r="E12" s="20" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="20" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C13" s="40" t="n">
         <v>3</v>
@@ -4731,12 +4739,12 @@
         <v>4</v>
       </c>
       <c r="E13" s="20" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="20" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C14" s="40" t="n">
         <v>10</v>
@@ -4766,7 +4774,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="41" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C19" s="47" t="n">
         <f aca="false">SUM(C6:C17)</f>
@@ -4779,7 +4787,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="28" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C20" s="48" t="n">
         <f aca="false">168-C19</f>
@@ -4792,7 +4800,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="17" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C22" s="49" t="n">
         <f aca="false">SUMIF(B6:B17,"Family*",D6:D17)-SUMIF(B6:B17,"Family*",C6:C17)</f>
@@ -4801,7 +4809,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="17" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C23" s="50" t="n">
         <f aca="false">C22*52</f>
@@ -4810,7 +4818,7 @@
     </row>
     <row r="25" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B25" s="32" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C25" s="32"/>
       <c r="D25" s="32"/>
@@ -4824,20 +4832,20 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B28" s="41" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C28" s="51" t="n">
         <f aca="false">'U · Understand'!C29</f>
         <v>12.0192307692308</v>
       </c>
       <c r="D28" s="32" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="E28" s="32"/>
     </row>
     <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="41" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C29" s="23" t="n">
         <f aca="false">MAX(0,SUMIF(B6:B17,"Paid work*",C6:C17)-SUMIF(B6:B17,"Paid work*",D6:D17))*52*C28</f>
@@ -4888,7 +4896,7 @@
   <sheetData>
     <row r="2" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="11" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C2" s="11"/>
       <c r="D2" s="11"/>
@@ -4900,7 +4908,7 @@
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="12" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C3" s="12"/>
       <c r="D3" s="12"/>
@@ -4912,45 +4920,45 @@
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="19" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C5" s="19" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="D5" s="19" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="E5" s="19" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="F5" s="19" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="G5" s="19" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="H5" s="19" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="I5" s="19" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C6" s="20" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="D6" s="20" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="E6" s="40" t="n">
         <v>0</v>
       </c>
       <c r="F6" s="20" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="G6" s="21" t="n">
         <v>150</v>
@@ -4960,24 +4968,24 @@
         <v>no time logged</v>
       </c>
       <c r="I6" s="20" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="20" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C7" s="20" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D7" s="20" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="E7" s="40" t="n">
         <v>3</v>
       </c>
       <c r="F7" s="20" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="G7" s="21" t="n">
         <v>60</v>
@@ -4987,18 +4995,18 @@
         <v>4.61538461538462</v>
       </c>
       <c r="I7" s="20" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="20" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C8" s="20" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="D8" s="20" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="E8" s="40" t="n">
         <v>0</v>
@@ -5012,7 +5020,7 @@
         <v/>
       </c>
       <c r="I8" s="20" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5186,7 +5194,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="28" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="G23" s="29" t="n">
         <f aca="false">SUMIF(C6:C21,"&lt;&gt;Career (raise/promotion)",G6:G21)</f>
@@ -5195,7 +5203,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="41" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="G24" s="23" t="n">
         <f aca="false">SUMIF(C6:C21,"Career (raise/promotion)",G6:G21)</f>
@@ -5204,7 +5212,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="41" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E25" s="53" t="n">
         <f aca="false">SUM(E6:E21)</f>
@@ -5213,7 +5221,7 @@
     </row>
     <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="17" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="G26" s="54" t="n">
         <f aca="false">IF('T · Track'!E58&gt;0,G23/'T · Track'!E58,0)</f>
@@ -5222,7 +5230,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B28" s="32" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C28" s="32"/>
       <c r="D28" s="32"/>
@@ -5277,7 +5285,7 @@
   <sheetData>
     <row r="2" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="11" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C2" s="11"/>
       <c r="D2" s="11"/>
@@ -5286,7 +5294,7 @@
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="12" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C3" s="12"/>
       <c r="D3" s="12"/>
@@ -5295,7 +5303,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="13" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5318,7 +5326,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="15" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C9" s="57" t="n">
         <f aca="false">IF(C14&lt;0,0,IF(C22&lt;C13,1,IF(C20&gt;0,2,IF(C22&lt;C23,3,IF(C25&lt;0.25*C13,4,IF(C25&lt;C13,5,6))))))</f>
@@ -5327,22 +5335,22 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="18" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="E11" s="18" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="15" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C12" s="58" t="n">
         <f aca="false">'T · Track'!E13</f>
         <v>2560</v>
       </c>
       <c r="E12" s="15" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="F12" s="59" t="n">
         <f aca="false">'U · Understand'!C29</f>
@@ -5351,14 +5359,14 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="15" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="C13" s="60" t="n">
         <f aca="false">'T · Track'!E58</f>
         <v>1740</v>
       </c>
       <c r="E13" s="15" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F13" s="61" t="n">
         <f aca="false">'U · Understand'!C31</f>
@@ -5367,14 +5375,14 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="15" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C14" s="61" t="n">
         <f aca="false">'T · Track'!E62</f>
         <v>555</v>
       </c>
       <c r="E14" s="15" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="F14" s="62" t="n">
         <f aca="false">'Income Streams'!E25</f>
@@ -5383,14 +5391,14 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="15" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C15" s="63" t="n">
         <f aca="false">'T · Track'!E63</f>
         <v>0.216796875</v>
       </c>
       <c r="E15" s="15" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="F15" s="64" t="n">
         <f aca="false">'Income Streams'!G26</f>
@@ -5399,14 +5407,14 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="15" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C16" s="65" t="n">
         <f aca="false">'T · Track'!E59</f>
         <v>265</v>
       </c>
       <c r="E16" s="15" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="F16" s="66" t="n">
         <f aca="false">'T · Time'!C22</f>
@@ -5415,14 +5423,14 @@
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="15" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C17" s="61" t="n">
         <f aca="false">'R · Reclaim'!F32</f>
         <v>48</v>
       </c>
       <c r="E17" s="15" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="F17" s="58" t="n">
         <f aca="false">'S · Save'!E32</f>
@@ -5431,14 +5439,14 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="15" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C18" s="61" t="n">
         <f aca="false">'R · Reclaim'!F33</f>
         <v>576</v>
       </c>
       <c r="E18" s="15" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="F18" s="61" t="n">
         <f aca="false">'Income Streams'!G24</f>
@@ -5447,106 +5455,106 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="18" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="15" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C20" s="65" t="n">
         <f aca="false">'U · Understand'!C17</f>
         <v>1500</v>
       </c>
       <c r="E20" s="67" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="15" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C21" s="65" t="n">
         <f aca="false">'U · Understand'!C19</f>
         <v>298.5</v>
       </c>
       <c r="E21" s="68" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="F21" s="68"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="15" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C22" s="61" t="n">
         <f aca="false">'S · Save'!C11</f>
         <v>1200</v>
       </c>
       <c r="E22" s="68" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="F22" s="68"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="15" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C23" s="60" t="n">
         <f aca="false">'S · Save'!C10</f>
         <v>5220</v>
       </c>
       <c r="E23" s="68" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="F23" s="68"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="15" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C24" s="63" t="n">
         <f aca="false">'S · Save'!C12</f>
         <v>0.229885057471264</v>
       </c>
       <c r="E24" s="68" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="F24" s="68"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="15" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C25" s="61" t="n">
         <f aca="false">'Income Streams'!G23</f>
         <v>60</v>
       </c>
       <c r="E25" s="68" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="F25" s="68"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E26" s="68" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="F26" s="68"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E27" s="68" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="F27" s="68"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="69" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="70" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Remove last name; frame debt and wealth story as own experience
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DDRxLznxQFLEsk2zkizz32
</commit_message>
<xml_diff>
--- a/icyber/TRUST-Tracker-Freedom-Edition.xlsx
+++ b/icyber/TRUST-Tracker-Freedom-Edition.xlsx
@@ -82,7 +82,7 @@
     <t xml:space="preserve">You work hard for your money. But is it creating the life you're working so hard for?</t>
   </si>
   <si>
-    <t xml:space="preserve">I'm a full-time cybersecurity consultant at a Big Four firm. I work a demanding job, and I'm supporting my mum after her cerebral haemorrhage. I paid off €20,000 of debt and I'm building wealth beside my career with the same system I share here. I don't teach this from the outside. I live it every week.</t>
+    <t xml:space="preserve">I'm a full-time cybersecurity consultant at a Big Four firm. I work a demanding job, and I'm supporting my mum after her cerebral haemorrhage. Everything here comes from my own experience: I paid off €20,000 of debt and I'm building wealth beside my career with the same system I share here. I don't teach this from the outside. I live it every week.</t>
   </si>
   <si>
     <t xml:space="preserve">You have a demanding career, bills to pay and people who depend on you. You earn a respectable income. Yet despite everything you do, you don't always feel as financially secure or independent as you thought you would.</t>
@@ -227,7 +227,7 @@
     <t xml:space="preserve">Money going out or still owed (debt)</t>
   </si>
   <si>
-    <t xml:space="preserve">© cybercnslt.com · Liliane Jörger · @cyber_cnslt · For personal use by the purchaser only, please don't resell or share.</t>
+    <t xml:space="preserve">© cybercnslt.com · Liliane · @cyber_cnslt · For personal use by the purchaser only, please don't resell or share.</t>
   </si>
   <si>
     <t xml:space="preserve">T · Track</t>
@@ -1880,7 +1880,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="48.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="3" t="s">
         <v>2</v>
       </c>

</xml_diff>

<commit_message>
Intro: mum receives care at home; balancing both alongside the 9-5
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DDRxLznxQFLEsk2zkizz32
</commit_message>
<xml_diff>
--- a/icyber/TRUST-Tracker-Freedom-Edition.xlsx
+++ b/icyber/TRUST-Tracker-Freedom-Edition.xlsx
@@ -82,7 +82,7 @@
     <t xml:space="preserve">You work hard for your money. But is it creating the life you're working so hard for?</t>
   </si>
   <si>
-    <t xml:space="preserve">I'm a full-time cybersecurity consultant at a Big Four firm. I work a demanding job, and I'm supporting my mum after her cerebral haemorrhage. Everything here comes from my own experience: I paid off €20,000 of debt and I'm building wealth beside my career with the same system I share here. I don't teach this from the outside. I live it every week.</t>
+    <t xml:space="preserve">I'm a full-time cybersecurity consultant at a Big Four firm. I work a demanding job, and alongside my 9–5 I support my mum, who receives care at home after her cerebral haemorrhage. Balancing both is demanding, so I know how little time is left at the end of the day. Everything here comes from my own experience: I paid off €20,000 of debt and I'm building wealth beside my career with the same system I share here. I don't teach this from the outside. I live it every week.</t>
   </si>
   <si>
     <t xml:space="preserve">You have a demanding career, bills to pay and people who depend on you. You earn a respectable income. Yet despite everything you do, you don't always feel as financially secure or independent as you thought you would.</t>
@@ -1880,7 +1880,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="78.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="3" t="s">
         <v>2</v>
       </c>

</xml_diff>

<commit_message>
Add compounding deep-dive page with chart; debt origins and scam story in intro
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DDRxLznxQFLEsk2zkizz32
</commit_message>
<xml_diff>
--- a/icyber/TRUST-Tracker-Freedom-Edition.xlsx
+++ b/icyber/TRUST-Tracker-Freedom-Edition.xlsx
@@ -91,7 +91,7 @@
     <t xml:space="preserve">How do I build a financially secure future without missing out on the people and moments that matter most today?</t>
   </si>
   <si>
-    <t xml:space="preserve">I know that feeling. I started as a flight attendant working toward becoming a pilot, until COVID changed those plans. I rebuilt my path in cybersecurity consulting. My income grew, but financial security didn't automatically follow. I paid off €20,000 of debt not by first earning more, but by understanding my finances and making deliberate changes.</t>
+    <t xml:space="preserve">I know that feeling. I started as a flight attendant working toward becoming a pilot, until COVID changed those plans. I rebuilt my path in cybersecurity consulting. My income grew, but financial security didn't automatically follow. In my 20s I took on loans for my study fees, made wrong financial decisions and even fell for an online scam. I paid off €20,000 of debt not by first earning more, but by understanding my finances and making deliberate changes. Now in my 30s, this is what I wish someone had told me in my 20s.</t>
   </si>
   <si>
     <t xml:space="preserve">WHY I REALLY BUILT THIS</t>
@@ -1922,7 +1922,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="93.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="4" t="s">
         <v>5</v>
       </c>

</xml_diff>

<commit_message>
Add trading story and 'only invest in what you understand' advice
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DDRxLznxQFLEsk2zkizz32
</commit_message>
<xml_diff>
--- a/icyber/TRUST-Tracker-Freedom-Edition.xlsx
+++ b/icyber/TRUST-Tracker-Freedom-Edition.xlsx
@@ -91,7 +91,7 @@
     <t xml:space="preserve">How do I build a financially secure future without missing out on the people and moments that matter most today?</t>
   </si>
   <si>
-    <t xml:space="preserve">I know that feeling. I started as a flight attendant working toward becoming a pilot, until COVID changed those plans. I rebuilt my path in cybersecurity consulting. My income grew, but financial security didn't automatically follow. In my 20s I took on loans for my study fees, made wrong financial decisions and even fell for an online scam. I paid off €20,000 of debt not by first earning more, but by understanding my finances and making deliberate changes. Now in my 30s, this is what I wish someone had told me in my 20s.</t>
+    <t xml:space="preserve">I know that feeling. I started as a flight attendant working toward becoming a pilot, until COVID changed those plans. I rebuilt my path in cybersecurity consulting. My income grew, but financial security didn't automatically follow. In my 20s I took on loans for my study fees, made wrong financial decisions and even fell for an online scam: I was heavily into trading without knowing much about it. My rule since then: only invest in what you understand. I paid off €20,000 of debt not by first earning more, but by understanding my finances and making deliberate changes. Now in my 30s, this is what I wish someone had told me in my 20s.</t>
   </si>
   <si>
     <t xml:space="preserve">WHY I REALLY BUILT THIS</t>
@@ -1922,7 +1922,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="93.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="108.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="4" t="s">
         <v>5</v>
       </c>

</xml_diff>

<commit_message>
Add wealth mindset and five laws of money (roadmap page 4, About Me)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DDRxLznxQFLEsk2zkizz32
</commit_message>
<xml_diff>
--- a/icyber/TRUST-Tracker-Freedom-Edition.xlsx
+++ b/icyber/TRUST-Tracker-Freedom-Edition.xlsx
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="297">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="351" uniqueCount="304">
   <si>
     <t xml:space="preserve">Hey, I'm Liliane.</t>
   </si>
@@ -149,6 +149,27 @@
   </si>
   <si>
     <t xml:space="preserve">Knowing your numbers is the beginning, not the goal. TRUST is the foundation for debt freedom, wealth building and additional income.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WEALTH STARTS WITH YOUR MINDSET</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Becoming wealthy starts with how you think about money and with understanding the laws of money. Money management is a skill you learn, not a talent you're born with.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 · Spend less than you earn. The gap is where all wealth begins.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 · Pay yourself first. Your future gets paid on payday, before bills and wants.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 · Protect what you have. A safety net and no expensive debt.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4 · Make your money work for you. Only invest in what you understand.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5 · Give it time. Compound growth rewards patience more than luck.</t>
   </si>
   <si>
     <t xml:space="preserve">YOUR NEXT STEP</t>
@@ -1889,7 +1910,7 @@
     <tabColor rgb="FF9E1B5E"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B2:B38"/>
+  <dimension ref="B2:B46"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
@@ -2032,19 +2053,54 @@
         <v>26</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B35" s="9" t="s">
+    <row r="34" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B34" s="4" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B36" s="10" t="s">
+    <row r="35" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B35" s="4" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B38" s="11" t="s">
+    <row r="36" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B36" s="4" t="s">
         <v>29</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B37" s="4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B38" s="4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B40" s="6" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B41" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B43" s="9" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B44" s="10" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B46" s="11" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -2079,7 +2135,7 @@
   <sheetData>
     <row r="2" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="12" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12"/>
@@ -2094,7 +2150,7 @@
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="13" t="s">
-        <v>265</v>
+        <v>272</v>
       </c>
       <c r="C3" s="13"/>
       <c r="D3" s="13"/>
@@ -2109,42 +2165,42 @@
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="20" t="s">
-        <v>266</v>
+        <v>273</v>
       </c>
       <c r="C5" s="20" t="s">
-        <v>267</v>
+        <v>274</v>
       </c>
       <c r="D5" s="20" t="s">
-        <v>268</v>
+        <v>275</v>
       </c>
       <c r="E5" s="20" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="F5" s="20" t="s">
-        <v>269</v>
+        <v>276</v>
       </c>
       <c r="G5" s="20" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="H5" s="20" t="s">
-        <v>270</v>
+        <v>277</v>
       </c>
       <c r="I5" s="20" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="J5" s="20" t="s">
-        <v>271</v>
+        <v>278</v>
       </c>
       <c r="K5" s="20" t="s">
-        <v>272</v>
+        <v>279</v>
       </c>
       <c r="L5" s="20" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="21" t="s">
-        <v>274</v>
+        <v>281</v>
       </c>
       <c r="C6" s="22" t="n">
         <v>2500</v>
@@ -2177,12 +2233,12 @@
         <v>Level 1 · Stable</v>
       </c>
       <c r="L6" s="21" t="s">
-        <v>275</v>
+        <v>282</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="21" t="s">
-        <v>276</v>
+        <v>283</v>
       </c>
       <c r="C7" s="22" t="n">
         <v>2560</v>
@@ -2215,7 +2271,7 @@
         <v>Level 1 · Stable</v>
       </c>
       <c r="L7" s="21" t="s">
-        <v>277</v>
+        <v>284</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2463,160 +2519,160 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>213</v>
+        <v>220</v>
       </c>
       <c r="E1" s="0" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
       <c r="F1" s="0" t="s">
-        <v>278</v>
+        <v>285</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>279</v>
+        <v>286</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>219</v>
+        <v>226</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>280</v>
+        <v>287</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>218</v>
+        <v>225</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>214</v>
+        <v>221</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>281</v>
+        <v>288</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>223</v>
+        <v>230</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>282</v>
+        <v>289</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>283</v>
+        <v>290</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>284</v>
+        <v>291</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>285</v>
+        <v>292</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>286</v>
+        <v>293</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>287</v>
+        <v>294</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>288</v>
+        <v>295</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>289</v>
+        <v>296</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>290</v>
+        <v>297</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>292</v>
+        <v>299</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>293</v>
+        <v>300</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>294</v>
+        <v>301</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>295</v>
+        <v>302</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>296</v>
+        <v>303</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>293</v>
+        <v>300</v>
       </c>
     </row>
   </sheetData>
@@ -2647,51 +2703,51 @@
   <sheetData>
     <row r="2" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="12" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="C2" s="12"/>
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="13" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="C3" s="13"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="14" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="15" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="15" t="s">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="15" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>38</v>
+        <v>45</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="15" t="s">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2700,23 +2756,23 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="14" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="15" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="15" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2725,31 +2781,31 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="14" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="17" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="C16" s="16" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="15" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="C17" s="16" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="18" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="C18" s="16" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2759,7 +2815,7 @@
     <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B20" s="15"/>
       <c r="C20" s="16" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
     </row>
   </sheetData>
@@ -2796,7 +2852,7 @@
   <sheetData>
     <row r="2" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="12" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12"/>
@@ -2805,7 +2861,7 @@
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="13" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="C3" s="13"/>
       <c r="D3" s="13"/>
@@ -2814,26 +2870,26 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="19" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="20" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="C6" s="20" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="E6" s="20" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="21" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="E7" s="22" t="n">
         <v>2500</v>
@@ -2841,10 +2897,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="21" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="C8" s="21" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="E8" s="23" t="n">
         <f aca="false">'Income Streams'!G23</f>
@@ -2853,10 +2909,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="21" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="C9" s="21" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="E9" s="22" t="n">
         <v>0</v>
@@ -2879,7 +2935,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="15" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="E13" s="24" t="n">
         <f aca="false">SUM(E7:E12)</f>
@@ -2888,52 +2944,52 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="19" t="s">
-        <v>67</v>
+        <v>74</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="20" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="C16" s="20" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="D16" s="20" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="E16" s="20" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="F16" s="20" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="21" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="C17" s="21" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="D17" s="21" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="E17" s="22" t="n">
         <v>900</v>
       </c>
       <c r="F17" s="21" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="21" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="C18" s="21" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="D18" s="21" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="E18" s="22" t="n">
         <v>140</v>
@@ -2942,13 +2998,13 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="21" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="C19" s="21" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="D19" s="21" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="E19" s="22" t="n">
         <v>320</v>
@@ -2957,13 +3013,13 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="21" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="C20" s="21" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="D20" s="21" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="E20" s="22" t="n">
         <v>90</v>
@@ -2972,13 +3028,13 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="21" t="s">
+        <v>87</v>
+      </c>
+      <c r="C21" s="21" t="s">
+        <v>87</v>
+      </c>
+      <c r="D21" s="21" t="s">
         <v>80</v>
-      </c>
-      <c r="C21" s="21" t="s">
-        <v>80</v>
-      </c>
-      <c r="D21" s="21" t="s">
-        <v>73</v>
       </c>
       <c r="E21" s="22" t="n">
         <v>80</v>
@@ -2987,13 +3043,13 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="21" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="C22" s="21" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="D22" s="21" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="E22" s="22" t="n">
         <v>150</v>
@@ -3002,13 +3058,13 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="21" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="C23" s="21" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="D23" s="21" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="E23" s="22" t="n">
         <v>60</v>
@@ -3017,13 +3073,13 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="21" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="C24" s="21" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="D24" s="21" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="E24" s="22" t="n">
         <v>45</v>
@@ -3032,13 +3088,13 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="21" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="C25" s="21" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="D25" s="21" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="E25" s="22" t="n">
         <v>120</v>
@@ -3047,13 +3103,13 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="21" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="C26" s="21" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="D26" s="21" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="E26" s="22" t="n">
         <v>100</v>
@@ -3272,7 +3328,7 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B58" s="15" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="E58" s="24" t="n">
         <f aca="false">SUMIF(D17:D56,"Need",E17:E56)</f>
@@ -3281,7 +3337,7 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B59" s="15" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="E59" s="24" t="n">
         <f aca="false">SUMIF(D17:D56,"Want",E17:E56)</f>
@@ -3290,7 +3346,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B60" s="25" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="E60" s="26" t="n">
         <f aca="false">SUMIF(C17:C56,"Caregiving",E17:E56)</f>
@@ -3299,7 +3355,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B61" s="27" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="E61" s="28" t="n">
         <f aca="false">SUM(E17:E56)-E58-E59</f>
@@ -3308,7 +3364,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B62" s="29" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="E62" s="30" t="n">
         <f aca="false">E13-E58-E59</f>
@@ -3317,7 +3373,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B63" s="29" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="E63" s="31" t="n">
         <f aca="false">IF(E13&gt;0,E62/E13,0)</f>
@@ -3369,7 +3425,7 @@
   <sheetData>
     <row r="2" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="12" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12"/>
@@ -3379,7 +3435,7 @@
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="13" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="C3" s="13"/>
       <c r="D3" s="13"/>
@@ -3389,33 +3445,33 @@
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="20" t="s">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="C5" s="20" t="s">
-        <v>101</v>
+        <v>108</v>
       </c>
       <c r="D5" s="20" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="E5" s="20" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="F5" s="20" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="G5" s="20" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="21" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="C6" s="22" t="n">
         <v>13</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="E6" s="22" t="n">
         <v>0</v>
@@ -3425,18 +3481,18 @@
         <v>13</v>
       </c>
       <c r="G6" s="21" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="21" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="C7" s="22" t="n">
         <v>35</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="E7" s="22" t="n">
         <v>15</v>
@@ -3446,18 +3502,18 @@
         <v>20</v>
       </c>
       <c r="G7" s="21" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="21" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="C8" s="22" t="n">
         <v>40</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="E8" s="22" t="n">
         <v>25</v>
@@ -3467,18 +3523,18 @@
         <v>15</v>
       </c>
       <c r="G8" s="21" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="21" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="C9" s="22" t="n">
         <v>3</v>
       </c>
       <c r="D9" s="21" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="E9" s="22" t="n">
         <v>3</v>
@@ -3722,7 +3778,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="15" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="F32" s="30" t="n">
         <f aca="false">SUM(F6:F30)</f>
@@ -3731,7 +3787,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="15" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="F33" s="30" t="n">
         <f aca="false">F32*12</f>
@@ -3740,7 +3796,7 @@
     </row>
     <row r="35" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B35" s="33" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="C35" s="33"/>
       <c r="D35" s="33"/>
@@ -3792,7 +3848,7 @@
   <sheetData>
     <row r="2" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="12" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12"/>
@@ -3804,7 +3860,7 @@
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="13" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="C3" s="13"/>
       <c r="D3" s="13"/>
@@ -3816,33 +3872,33 @@
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="20" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="C5" s="20" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="D5" s="20" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="E5" s="20" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="F5" s="20" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="G5" s="20" t="s">
-        <v>127</v>
+        <v>134</v>
       </c>
       <c r="H5" s="20" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="I5" s="20" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="21" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="C6" s="22" t="n">
         <v>1500</v>
@@ -3871,7 +3927,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="21" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="C7" s="22" t="n">
         <v>0</v>
@@ -4052,14 +4108,14 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="15" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="C17" s="38" t="n">
         <f aca="false">SUM(C6:C15)</f>
         <v>1500</v>
       </c>
       <c r="D17" s="33" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="E17" s="33"/>
       <c r="F17" s="33"/>
@@ -4069,7 +4125,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="15" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="C18" s="39" t="n">
         <f aca="false">SUM(G6:G15)</f>
@@ -4084,7 +4140,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="15" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="C19" s="38" t="n">
         <f aca="false">C18*12</f>
@@ -4099,27 +4155,27 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="19" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B23" s="20" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="C23" s="20" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B24" s="16" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="C24" s="40" t="n">
         <f aca="false">'T · Track'!E7</f>
         <v>2500</v>
       </c>
       <c r="D24" s="33" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="E24" s="33"/>
       <c r="F24" s="33"/>
@@ -4129,7 +4185,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="16" t="s">
-        <v>141</v>
+        <v>148</v>
       </c>
       <c r="C25" s="41" t="n">
         <v>39</v>
@@ -4143,7 +4199,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="16" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="C26" s="41" t="n">
         <v>4</v>
@@ -4157,7 +4213,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="16" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
       <c r="C27" s="41" t="n">
         <v>5</v>
@@ -4171,7 +4227,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="42" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="C28" s="43" t="n">
         <f aca="false">(N(C25)+N(C26)+N(C27))*52/12</f>
@@ -4186,14 +4242,14 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B29" s="29" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="C29" s="44" t="n">
         <f aca="false">IF(C28&gt;0,C24/C28,0)</f>
         <v>12.0192307692308</v>
       </c>
       <c r="D29" s="33" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="E29" s="33"/>
       <c r="F29" s="33"/>
@@ -4203,7 +4259,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="16" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="C30" s="45" t="n">
         <v>21</v>
@@ -4217,7 +4273,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="29" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="C31" s="30" t="n">
         <f aca="false">C29*N(C30)</f>
@@ -4268,7 +4324,7 @@
   <sheetData>
     <row r="2" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="12" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12"/>
@@ -4278,7 +4334,7 @@
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="13" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="C3" s="13"/>
       <c r="D3" s="13"/>
@@ -4288,27 +4344,27 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="19" t="s">
-        <v>151</v>
+        <v>158</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="20" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="C6" s="20" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="16" t="s">
-        <v>152</v>
+        <v>159</v>
       </c>
       <c r="C7" s="40" t="n">
         <f aca="false">'T · Track'!E58</f>
         <v>1740</v>
       </c>
       <c r="D7" s="33" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
       <c r="E7" s="33"/>
       <c r="F7" s="33"/>
@@ -4316,7 +4372,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="16" t="s">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="C8" s="45" t="n">
         <v>3</v>
@@ -4328,7 +4384,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="42" t="s">
-        <v>155</v>
+        <v>162</v>
       </c>
       <c r="C9" s="46" t="n">
         <f aca="false">C7</f>
@@ -4341,7 +4397,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="42" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="C10" s="24" t="n">
         <f aca="false">C7*N(C8)</f>
@@ -4354,7 +4410,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="16" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="C11" s="22" t="n">
         <v>1200</v>
@@ -4362,7 +4418,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="29" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="C12" s="31" t="n">
         <f aca="false">IF(C10&gt;0,MIN(1,N(C11)/C10),0)</f>
@@ -4371,7 +4427,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="16" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="C13" s="22" t="n">
         <v>250</v>
@@ -4379,7 +4435,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="42" t="s">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="C14" s="36" t="n">
         <f aca="false">IF(N(C11)&gt;=C10,"Done ✓",IF(N(C13)&gt;0,ROUNDUP((C10-N(C11))/C13,0),"Add a transfer"))</f>
@@ -4388,32 +4444,32 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="19" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B18" s="20" t="s">
-        <v>162</v>
+        <v>169</v>
       </c>
       <c r="C18" s="20" t="s">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="D18" s="20" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="E18" s="20" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="F18" s="20" t="s">
+        <v>172</v>
+      </c>
+      <c r="G18" s="20" t="s">
         <v>165</v>
-      </c>
-      <c r="G18" s="20" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="21" t="s">
-        <v>166</v>
+        <v>173</v>
       </c>
       <c r="C19" s="22" t="n">
         <v>1500</v>
@@ -4435,7 +4491,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="21" t="s">
-        <v>167</v>
+        <v>174</v>
       </c>
       <c r="C20" s="22" t="n">
         <v>600</v>
@@ -4457,7 +4513,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="21" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="C21" s="22" t="n">
         <v>1800</v>
@@ -4577,7 +4633,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="42" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
       <c r="E30" s="24" t="n">
         <f aca="false">SUM(E19:E28)</f>
@@ -4586,7 +4642,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="29" t="s">
-        <v>170</v>
+        <v>177</v>
       </c>
       <c r="E31" s="30" t="n">
         <f aca="false">N(C13)+E30</f>
@@ -4595,7 +4651,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="15" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="E32" s="24" t="n">
         <f aca="false">'T · Track'!E62-E31</f>
@@ -4604,7 +4660,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B33" s="33" t="s">
-        <v>172</v>
+        <v>179</v>
       </c>
       <c r="C33" s="33"/>
       <c r="D33" s="33"/>
@@ -4646,7 +4702,7 @@
   <sheetData>
     <row r="2" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="12" t="s">
-        <v>173</v>
+        <v>180</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12"/>
@@ -4654,7 +4710,7 @@
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="13" t="s">
-        <v>174</v>
+        <v>181</v>
       </c>
       <c r="C3" s="13"/>
       <c r="D3" s="13"/>
@@ -4662,21 +4718,21 @@
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="20" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
       <c r="C5" s="20" t="s">
-        <v>176</v>
+        <v>183</v>
       </c>
       <c r="D5" s="20" t="s">
-        <v>177</v>
+        <v>184</v>
       </c>
       <c r="E5" s="20" t="s">
-        <v>178</v>
+        <v>185</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="21" t="s">
-        <v>179</v>
+        <v>186</v>
       </c>
       <c r="C6" s="41" t="n">
         <v>49</v>
@@ -4685,12 +4741,12 @@
         <v>52</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>180</v>
+        <v>187</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="21" t="s">
-        <v>181</v>
+        <v>188</v>
       </c>
       <c r="C7" s="41" t="n">
         <v>43</v>
@@ -4699,12 +4755,12 @@
         <v>40</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>182</v>
+        <v>189</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="21" t="s">
-        <v>183</v>
+        <v>190</v>
       </c>
       <c r="C8" s="41" t="n">
         <v>5</v>
@@ -4716,7 +4772,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="21" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="C9" s="41" t="n">
         <v>10</v>
@@ -4725,12 +4781,12 @@
         <v>10</v>
       </c>
       <c r="E9" s="21" t="s">
-        <v>184</v>
+        <v>191</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="21" t="s">
-        <v>185</v>
+        <v>192</v>
       </c>
       <c r="C10" s="41" t="n">
         <v>10</v>
@@ -4739,12 +4795,12 @@
         <v>8</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>186</v>
+        <v>193</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="21" t="s">
-        <v>187</v>
+        <v>194</v>
       </c>
       <c r="C11" s="41" t="n">
         <v>12</v>
@@ -4753,12 +4809,12 @@
         <v>16</v>
       </c>
       <c r="E11" s="21" t="s">
-        <v>188</v>
+        <v>195</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="21" t="s">
-        <v>189</v>
+        <v>196</v>
       </c>
       <c r="C12" s="41" t="n">
         <v>3</v>
@@ -4767,12 +4823,12 @@
         <v>4</v>
       </c>
       <c r="E12" s="21" t="s">
-        <v>190</v>
+        <v>197</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="21" t="s">
-        <v>191</v>
+        <v>198</v>
       </c>
       <c r="C13" s="41" t="n">
         <v>3</v>
@@ -4781,12 +4837,12 @@
         <v>4</v>
       </c>
       <c r="E13" s="21" t="s">
-        <v>192</v>
+        <v>199</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="21" t="s">
-        <v>193</v>
+        <v>200</v>
       </c>
       <c r="C14" s="41" t="n">
         <v>10</v>
@@ -4816,7 +4872,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="42" t="s">
-        <v>194</v>
+        <v>201</v>
       </c>
       <c r="C19" s="48" t="n">
         <f aca="false">SUM(C6:C17)</f>
@@ -4829,7 +4885,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="29" t="s">
-        <v>195</v>
+        <v>202</v>
       </c>
       <c r="C20" s="49" t="n">
         <f aca="false">168-C19</f>
@@ -4842,7 +4898,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="18" t="s">
-        <v>196</v>
+        <v>203</v>
       </c>
       <c r="C22" s="50" t="n">
         <f aca="false">SUMIF(B6:B17,"Family*",D6:D17)-SUMIF(B6:B17,"Family*",C6:C17)</f>
@@ -4851,7 +4907,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="18" t="s">
-        <v>197</v>
+        <v>204</v>
       </c>
       <c r="C23" s="51" t="n">
         <f aca="false">C22*52</f>
@@ -4860,7 +4916,7 @@
     </row>
     <row r="25" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B25" s="33" t="s">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="C25" s="33"/>
       <c r="D25" s="33"/>
@@ -4874,20 +4930,20 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B28" s="42" t="s">
-        <v>199</v>
+        <v>206</v>
       </c>
       <c r="C28" s="52" t="n">
         <f aca="false">'U · Understand'!C29</f>
         <v>12.0192307692308</v>
       </c>
       <c r="D28" s="33" t="s">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="E28" s="33"/>
     </row>
     <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="42" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="C29" s="24" t="n">
         <f aca="false">MAX(0,SUMIF(B6:B17,"Paid work*",C6:C17)-SUMIF(B6:B17,"Paid work*",D6:D17))*52*C28</f>
@@ -4938,7 +4994,7 @@
   <sheetData>
     <row r="2" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="12" t="s">
-        <v>202</v>
+        <v>209</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12"/>
@@ -4950,7 +5006,7 @@
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="13" t="s">
-        <v>203</v>
+        <v>210</v>
       </c>
       <c r="C3" s="13"/>
       <c r="D3" s="13"/>
@@ -4962,45 +5018,45 @@
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="20" t="s">
-        <v>204</v>
+        <v>211</v>
       </c>
       <c r="C5" s="20" t="s">
-        <v>205</v>
+        <v>212</v>
       </c>
       <c r="D5" s="20" t="s">
-        <v>206</v>
+        <v>213</v>
       </c>
       <c r="E5" s="20" t="s">
-        <v>207</v>
+        <v>214</v>
       </c>
       <c r="F5" s="20" t="s">
-        <v>208</v>
+        <v>215</v>
       </c>
       <c r="G5" s="20" t="s">
-        <v>209</v>
+        <v>216</v>
       </c>
       <c r="H5" s="20" t="s">
-        <v>210</v>
+        <v>217</v>
       </c>
       <c r="I5" s="20" t="s">
-        <v>211</v>
+        <v>218</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="21" t="s">
-        <v>212</v>
+        <v>219</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>213</v>
+        <v>220</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>214</v>
+        <v>221</v>
       </c>
       <c r="E6" s="41" t="n">
         <v>0</v>
       </c>
       <c r="F6" s="21" t="s">
-        <v>215</v>
+        <v>222</v>
       </c>
       <c r="G6" s="22" t="n">
         <v>150</v>
@@ -5010,24 +5066,24 @@
         <v>no time logged</v>
       </c>
       <c r="I6" s="21" t="s">
-        <v>216</v>
+        <v>223</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="21" t="s">
-        <v>217</v>
+        <v>224</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>218</v>
+        <v>225</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>219</v>
+        <v>226</v>
       </c>
       <c r="E7" s="41" t="n">
         <v>3</v>
       </c>
       <c r="F7" s="21" t="s">
-        <v>220</v>
+        <v>227</v>
       </c>
       <c r="G7" s="22" t="n">
         <v>60</v>
@@ -5037,18 +5093,18 @@
         <v>4.61538461538462</v>
       </c>
       <c r="I7" s="21" t="s">
-        <v>221</v>
+        <v>228</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="21" t="s">
-        <v>222</v>
+        <v>229</v>
       </c>
       <c r="C8" s="21" t="s">
-        <v>223</v>
+        <v>230</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
       <c r="E8" s="41" t="n">
         <v>0</v>
@@ -5062,7 +5118,7 @@
         <v/>
       </c>
       <c r="I8" s="21" t="s">
-        <v>225</v>
+        <v>232</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5236,7 +5292,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="29" t="s">
-        <v>226</v>
+        <v>233</v>
       </c>
       <c r="G23" s="30" t="n">
         <f aca="false">SUMIF(C6:C21,"&lt;&gt;Career (raise/promotion)",G6:G21)</f>
@@ -5245,7 +5301,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="42" t="s">
-        <v>227</v>
+        <v>234</v>
       </c>
       <c r="G24" s="24" t="n">
         <f aca="false">SUMIF(C6:C21,"Career (raise/promotion)",G6:G21)</f>
@@ -5254,7 +5310,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="42" t="s">
-        <v>228</v>
+        <v>235</v>
       </c>
       <c r="E25" s="54" t="n">
         <f aca="false">SUM(E6:E21)</f>
@@ -5263,7 +5319,7 @@
     </row>
     <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="18" t="s">
-        <v>229</v>
+        <v>236</v>
       </c>
       <c r="G26" s="55" t="n">
         <f aca="false">IF('T · Track'!E58&gt;0,G23/'T · Track'!E58,0)</f>
@@ -5272,7 +5328,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B28" s="33" t="s">
-        <v>230</v>
+        <v>237</v>
       </c>
       <c r="C28" s="33"/>
       <c r="D28" s="33"/>
@@ -5327,7 +5383,7 @@
   <sheetData>
     <row r="2" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="12" t="s">
-        <v>231</v>
+        <v>238</v>
       </c>
       <c r="C2" s="12"/>
       <c r="D2" s="12"/>
@@ -5336,7 +5392,7 @@
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="13" t="s">
-        <v>232</v>
+        <v>239</v>
       </c>
       <c r="C3" s="13"/>
       <c r="D3" s="13"/>
@@ -5345,7 +5401,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="14" t="s">
-        <v>233</v>
+        <v>240</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5368,7 +5424,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="16" t="s">
-        <v>234</v>
+        <v>241</v>
       </c>
       <c r="C9" s="58" t="n">
         <f aca="false">IF(C14&lt;0,0,IF(C22&lt;C13,1,IF(C20&gt;0,2,IF(C22&lt;C23,3,IF(C25&lt;0.25*C13,4,IF(C25&lt;C13,5,6))))))</f>
@@ -5377,22 +5433,22 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="19" t="s">
-        <v>235</v>
+        <v>242</v>
       </c>
       <c r="E11" s="19" t="s">
-        <v>236</v>
+        <v>243</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="16" t="s">
-        <v>237</v>
+        <v>244</v>
       </c>
       <c r="C12" s="59" t="n">
         <f aca="false">'T · Track'!E13</f>
         <v>2560</v>
       </c>
       <c r="E12" s="16" t="s">
-        <v>238</v>
+        <v>245</v>
       </c>
       <c r="F12" s="60" t="n">
         <f aca="false">'U · Understand'!C29</f>
@@ -5401,14 +5457,14 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="16" t="s">
-        <v>239</v>
+        <v>246</v>
       </c>
       <c r="C13" s="61" t="n">
         <f aca="false">'T · Track'!E58</f>
         <v>1740</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="F13" s="62" t="n">
         <f aca="false">'U · Understand'!C31</f>
@@ -5417,14 +5473,14 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="16" t="s">
-        <v>240</v>
+        <v>247</v>
       </c>
       <c r="C14" s="62" t="n">
         <f aca="false">'T · Track'!E62</f>
         <v>555</v>
       </c>
       <c r="E14" s="16" t="s">
-        <v>241</v>
+        <v>248</v>
       </c>
       <c r="F14" s="63" t="n">
         <f aca="false">'Income Streams'!E25</f>
@@ -5433,14 +5489,14 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="16" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="C15" s="64" t="n">
         <f aca="false">'T · Track'!E63</f>
         <v>0.216796875</v>
       </c>
       <c r="E15" s="16" t="s">
-        <v>242</v>
+        <v>249</v>
       </c>
       <c r="F15" s="65" t="n">
         <f aca="false">'Income Streams'!G26</f>
@@ -5449,14 +5505,14 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="16" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="C16" s="66" t="n">
         <f aca="false">'T · Track'!E59</f>
         <v>265</v>
       </c>
       <c r="E16" s="16" t="s">
-        <v>243</v>
+        <v>250</v>
       </c>
       <c r="F16" s="67" t="n">
         <f aca="false">'T · Time'!C22</f>
@@ -5465,14 +5521,14 @@
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="16" t="s">
-        <v>244</v>
+        <v>251</v>
       </c>
       <c r="C17" s="62" t="n">
         <f aca="false">'R · Reclaim'!F32</f>
         <v>48</v>
       </c>
       <c r="E17" s="16" t="s">
-        <v>245</v>
+        <v>252</v>
       </c>
       <c r="F17" s="59" t="n">
         <f aca="false">'S · Save'!E32</f>
@@ -5481,14 +5537,14 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="16" t="s">
-        <v>246</v>
+        <v>253</v>
       </c>
       <c r="C18" s="62" t="n">
         <f aca="false">'R · Reclaim'!F33</f>
         <v>576</v>
       </c>
       <c r="E18" s="16" t="s">
-        <v>247</v>
+        <v>254</v>
       </c>
       <c r="F18" s="62" t="n">
         <f aca="false">'Income Streams'!G24</f>
@@ -5497,106 +5553,106 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="19" t="s">
-        <v>248</v>
+        <v>255</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="16" t="s">
-        <v>249</v>
+        <v>256</v>
       </c>
       <c r="C20" s="66" t="n">
         <f aca="false">'U · Understand'!C17</f>
         <v>1500</v>
       </c>
       <c r="E20" s="68" t="s">
-        <v>250</v>
+        <v>257</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="16" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="C21" s="66" t="n">
         <f aca="false">'U · Understand'!C19</f>
         <v>298.5</v>
       </c>
       <c r="E21" s="69" t="s">
-        <v>251</v>
+        <v>258</v>
       </c>
       <c r="F21" s="69"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="16" t="s">
-        <v>252</v>
+        <v>259</v>
       </c>
       <c r="C22" s="62" t="n">
         <f aca="false">'S · Save'!C11</f>
         <v>1200</v>
       </c>
       <c r="E22" s="69" t="s">
-        <v>253</v>
+        <v>260</v>
       </c>
       <c r="F22" s="69"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="16" t="s">
-        <v>254</v>
+        <v>261</v>
       </c>
       <c r="C23" s="61" t="n">
         <f aca="false">'S · Save'!C10</f>
         <v>5220</v>
       </c>
       <c r="E23" s="69" t="s">
-        <v>255</v>
+        <v>262</v>
       </c>
       <c r="F23" s="69"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="16" t="s">
-        <v>256</v>
+        <v>263</v>
       </c>
       <c r="C24" s="64" t="n">
         <f aca="false">'S · Save'!C12</f>
         <v>0.229885057471264</v>
       </c>
       <c r="E24" s="69" t="s">
-        <v>257</v>
+        <v>264</v>
       </c>
       <c r="F24" s="69"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="16" t="s">
-        <v>258</v>
+        <v>265</v>
       </c>
       <c r="C25" s="62" t="n">
         <f aca="false">'Income Streams'!G23</f>
         <v>60</v>
       </c>
       <c r="E25" s="69" t="s">
-        <v>259</v>
+        <v>266</v>
       </c>
       <c r="F25" s="69"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E26" s="69" t="s">
-        <v>260</v>
+        <v>267</v>
       </c>
       <c r="F26" s="69"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E27" s="69" t="s">
-        <v>261</v>
+        <v>268</v>
       </c>
       <c r="F27" s="69"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="70" t="s">
-        <v>262</v>
+        <v>269</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="71" t="s">
-        <v>263</v>
+        <v>270</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Debt paid off: €30,000
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DDRxLznxQFLEsk2zkizz32
</commit_message>
<xml_diff>
--- a/icyber/TRUST-Tracker-Freedom-Edition.xlsx
+++ b/icyber/TRUST-Tracker-Freedom-Edition.xlsx
@@ -82,7 +82,7 @@
     <t xml:space="preserve">You work hard for your money. But is it creating the life you're working so hard for?</t>
   </si>
   <si>
-    <t xml:space="preserve">I'm a full-time cybersecurity consultant at a Big Four firm. I work a demanding job, and alongside my 9–5 I support my mum, who receives care at home after her cerebral haemorrhage. Balancing both is demanding, so I know how little time is left at the end of the day. Everything here comes from my own experience: I paid off €20,000 of debt and I'm building wealth beside my career with the same system I share here. I don't teach this from the outside. I've experienced it myself.</t>
+    <t xml:space="preserve">I'm a full-time cybersecurity consultant at a Big Four firm. I work a demanding job, and alongside my 9–5 I support my mum, who receives care at home after her cerebral haemorrhage. Balancing both is demanding, so I know how little time is left at the end of the day. Everything here comes from my own experience: I paid off €30,000 of debt and I'm building wealth beside my career with the same system I share here. I don't teach this from the outside. I've experienced it myself.</t>
   </si>
   <si>
     <t xml:space="preserve">You have a demanding career, bills to pay and people who depend on you. You earn a respectable income. Yet despite everything you do, you don't always feel as financially secure or independent as you thought you would.</t>
@@ -91,7 +91,7 @@
     <t xml:space="preserve">How do I build a financially secure future without missing out on the people and moments that matter most today?</t>
   </si>
   <si>
-    <t xml:space="preserve">I know that feeling. I started as a flight attendant working toward becoming a pilot, until COVID changed those plans. I rebuilt my path in cybersecurity consulting. My income grew, but financial security didn't automatically follow. In my 20s I took on loans for my study fees, made wrong financial decisions and even fell for an online scam: I was heavily into trading without knowing much about it. My rule since then: only invest in what you understand. I paid off €20,000 of debt not by first earning more, but by understanding my finances and making deliberate changes. Now in my 30s, this is what I wish someone had told me in my 20s.</t>
+    <t xml:space="preserve">I know that feeling. I started as a flight attendant working toward becoming a pilot, until COVID changed those plans. I rebuilt my path in cybersecurity consulting. My income grew, but financial security didn't automatically follow. In my 20s I took on loans for my study fees, made wrong financial decisions and even fell for an online scam: I was heavily into trading without knowing much about it. My rule since then: only invest in what you understand. I paid off €30,000 of debt not by first earning more, but by understanding my finances and making deliberate changes. Now in my 30s, this is what I wish someone had told me in my 20s.</t>
   </si>
   <si>
     <t xml:space="preserve">WHY I REALLY BUILT THIS</t>

</xml_diff>

<commit_message>
Why section: overtime, corporate ladder, what true success means
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DDRxLznxQFLEsk2zkizz32
</commit_message>
<xml_diff>
--- a/icyber/TRUST-Tracker-Freedom-Edition.xlsx
+++ b/icyber/TRUST-Tracker-Freedom-Edition.xlsx
@@ -97,7 +97,7 @@
     <t xml:space="preserve">WHY I REALLY BUILT THIS</t>
   </si>
   <si>
-    <t xml:space="preserve">My mum is 83. When she had her cerebral haemorrhage, I realised how valuable time really is, and how little of it I had left after work. I want to spend as much time with her as I possibly can. Not someday, but now.</t>
+    <t xml:space="preserve">My mum is 83. When she had her cerebral haemorrhage, I realised how valuable time really is, and how little of it I had left. For years I worked long hours and stayed late almost every single day, because I believed climbing the corporate ladder was what success meant. But true success is realising what truly matters in life, and then taking the steps, one by one, that lead you there. We only get this one life. I want to spend as much time with her as I possibly can. Not someday, but now.</t>
   </si>
   <si>
     <t xml:space="preserve">Every plan I found told me to quit my job or hustle harder. None were made for someone with a demanding career and a parent who needs them. I wished I'd had a clear, honest plan for the few hours I actually had. So I built it for myself. You shouldn't need a wake-up call to start.</t>
@@ -1953,7 +1953,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="48.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="93.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="7" t="s">
         <v>7</v>
       </c>

</xml_diff>

<commit_message>
Why section: quitting/hustle plans risk financial security
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DDRxLznxQFLEsk2zkizz32
</commit_message>
<xml_diff>
--- a/icyber/TRUST-Tracker-Freedom-Edition.xlsx
+++ b/icyber/TRUST-Tracker-Freedom-Edition.xlsx
@@ -100,7 +100,7 @@
     <t xml:space="preserve">My mum is 83. When she had her cerebral haemorrhage, I realised how valuable time really is, and how little of it I had left. For years I worked long hours and stayed late almost every single day, because I believed climbing the corporate ladder was what success meant. But true success is realising what truly matters in life, and then taking the steps, one by one, that lead you there. We only get this one life. I want to spend as much time with her as I possibly can. Not someday, but now.</t>
   </si>
   <si>
-    <t xml:space="preserve">Every plan I found told me to quit my job or hustle harder. None were made for someone with a demanding career and a parent who needs them. I wished I'd had a clear, honest plan for the few hours I actually had. So I built it for myself. You shouldn't need a wake-up call to start.</t>
+    <t xml:space="preserve">Every plan I found told me to quit my job, hustle harder or get rich fast. That's unrealistic unless you're willing to risk your financial security, and when people depend on you, that's not a risk worth taking. None were made for someone with a demanding career and a parent who needs them. I wished I'd had a clear, honest plan for the few hours I actually had. So I built it for myself. You shouldn't need a wake-up call to start.</t>
   </si>
   <si>
     <t xml:space="preserve">That's why I created the TRUST Sheet. No judgment. No unrealistic promises. No complicated jargon. Just a practical starting point for making your money work toward the life you actually want.</t>
@@ -1958,7 +1958,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="48.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="78.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="4" t="s">
         <v>8</v>
       </c>

</xml_diff>

<commit_message>
Why section: hours left when not exhausted
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DDRxLznxQFLEsk2zkizz32
</commit_message>
<xml_diff>
--- a/icyber/TRUST-Tracker-Freedom-Edition.xlsx
+++ b/icyber/TRUST-Tracker-Freedom-Edition.xlsx
@@ -100,7 +100,7 @@
     <t xml:space="preserve">My mum is 83. When she had her cerebral haemorrhage, I realised how valuable time really is, and how little of it I had left. For years I worked long hours and stayed late almost every single day, because I believed climbing the corporate ladder was what success meant. But true success is realising what truly matters in life, and then taking the steps, one by one, that lead you there. We only get this one life. I want to spend as much time with her as I possibly can. Not someday, but now.</t>
   </si>
   <si>
-    <t xml:space="preserve">Most of the financial advice out there told me to quit my job, hustle harder or get rich fast. That's unrealistic unless you're willing to risk your financial security, and when people depend on you, that's not a risk worth taking. None were made for someone with a demanding career and a mum who needs them. I wished I'd had a clear, honest plan for the few hours I actually had. So I built it for myself. You shouldn't need a wake-up call to start.</t>
+    <t xml:space="preserve">Most of the financial advice out there told me to quit my job, hustle harder or get rich fast. That's unrealistic unless you're willing to risk your financial security, and when people depend on you, that's not a risk worth taking. None were made for someone with a demanding career and a mum who needs them. I wished I'd had a clear, honest plan for the few hours I actually had left, when I wasn't already exhausted from work and every other responsibility around me. So I built it for myself. You shouldn't need a wake-up call to start.</t>
   </si>
   <si>
     <t xml:space="preserve">That's why I created the TRUST Sheet. No judgment. No unrealistic promises. No complicated jargon. Just a practical starting point for making your money work toward the life you actually want.</t>
@@ -1958,7 +1958,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="78.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="93.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="4" t="s">
         <v>8</v>
       </c>

</xml_diff>